<commit_message>
feat(whatsapp): dispatch test messages to test staff registry and record meta wamid audit log
</commit_message>
<xml_diff>
--- a/Test_Teachers_And_Staff_Registry.xlsx
+++ b/Test_Teachers_And_Staff_Registry.xlsx
@@ -1,122 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet sheetId="1" name="Test_Staff_Registry" state="visible" r:id="rId4"/>
+    <sheet name="Test_Staff_Registry" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
-  <si>
-    <t>S.No</t>
-  </si>
-  <si>
-    <t>Teacher / Staff Name</t>
-  </si>
-  <si>
-    <t>Mobile Number (10 Digit)</t>
-  </si>
-  <si>
-    <t>Designation / Subject</t>
-  </si>
-  <si>
-    <t>School / College</t>
-  </si>
-  <si>
-    <t>Email Address</t>
-  </si>
-  <si>
-    <t>WhatsApp Status</t>
-  </si>
-  <si>
-    <t>Last Dispatch Date</t>
-  </si>
-  <si>
-    <t>Notes / Verification Status</t>
-  </si>
-  <si>
-    <t>TEST OBSERVER 1</t>
-  </si>
-  <si>
-    <t>EXAM COORDINATOR</t>
-  </si>
-  <si>
-    <t>MEENA SHAH MEMORIAL SCHOOL</t>
-  </si>
-  <si>
-    <t>coordinator@meenashah.edu</t>
-  </si>
-  <si>
-    <t>PENDING</t>
-  </si>
-  <si>
-    <t>Primary verification test recipient</t>
-  </si>
-  <si>
-    <t>TEST OBSERVER 2</t>
-  </si>
-  <si>
-    <t>HEAD TEACHER / INVIGILATOR</t>
-  </si>
-  <si>
-    <t>teacher@meenashah.edu</t>
-  </si>
-  <si>
-    <t>Secondary verification test recipient</t>
-  </si>
-  <si>
-    <t>ADMIN PORTAL CONTROLLER</t>
-  </si>
-  <si>
-    <t>PORTAL CONTROLLER</t>
-  </si>
-  <si>
-    <t>tabrezaalam92@gmail.com</t>
-  </si>
-  <si>
-    <t>Registered sender / admin phone</t>
-  </si>
-  <si>
-    <t>DR. RAMESH SHARMA</t>
-  </si>
-  <si>
-    <t>SENIOR EVALUATOR</t>
-  </si>
-  <si>
-    <t>MEENA SHAH PUBLIC SCHOOL</t>
-  </si>
-  <si>
-    <t>Added for examination test dispatch</t>
-  </si>
-  <si>
-    <t>AJAY SIR</t>
-  </si>
-  <si>
-    <t>DEAN MSITM COLLEGE</t>
-  </si>
-  <si>
-    <t>SAEED SIR (baba ji)</t>
-  </si>
-  <si>
-    <t>Manager</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -140,21 +65,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -479,182 +396,211 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="9.285714285714286" customWidth="1"/>
-    <col min="2" max="2" width="28.857142857142858" customWidth="1"/>
-    <col min="3" max="3" width="25.857142857142858" customWidth="1"/>
-    <col min="4" max="4" width="30.857142857142858" customWidth="1"/>
-    <col min="5" max="5" width="35.857142857142854" customWidth="1"/>
-    <col min="6" max="6" width="28.857142857142858" customWidth="1"/>
-    <col min="7" max="7" width="18.857142857142858" customWidth="1"/>
-    <col min="8" max="8" width="24.857142857142858" customWidth="1"/>
-    <col min="9" max="9" width="35.857142857142854" customWidth="1"/>
-    <col min="10" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="35.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>S.No</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Teacher / Staff Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Mobile Number (10 Digit)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Designation / Subject</v>
+      </c>
+      <c r="E1" t="str">
+        <v>School / College</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Email Address</v>
+      </c>
+      <c r="G1" t="str">
+        <v>WhatsApp Status</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Notes / Verification Status</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Last Dispatch Date</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>9</v>
+      <c r="B2" t="str">
+        <v>TEST OBSERVER 1</v>
       </c>
       <c r="C2">
         <v>918948905711</v>
       </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>14</v>
+      <c r="D2" t="str">
+        <v>EXAM COORDINATOR</v>
+      </c>
+      <c r="E2" t="str">
+        <v>MEENA SHAH MEMORIAL SCHOOL</v>
+      </c>
+      <c r="F2" t="str">
+        <v>coordinator@meenashah.edu</v>
+      </c>
+      <c r="G2" t="str">
+        <v>SENT</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Delivered via ICPaaS (Meta ID: wamid.HBgMOTE4OTQ4OTA1NzExFQIAERgSOEUyMDg1ODg4MTg1QTk3MDlDAA==)</v>
+      </c>
+      <c r="I2" t="str">
+        <v>23/10/2026, 3:33:03 pm</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>15</v>
+      <c r="B3" t="str">
+        <v>TEST OBSERVER 2</v>
       </c>
       <c r="C3">
         <v>919795600217</v>
       </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" t="s">
-        <v>18</v>
+      <c r="D3" t="str">
+        <v>HEAD TEACHER / INVIGILATOR</v>
+      </c>
+      <c r="E3" t="str">
+        <v>MEENA SHAH MEMORIAL SCHOOL</v>
+      </c>
+      <c r="F3" t="str">
+        <v>teacher@meenashah.edu</v>
+      </c>
+      <c r="G3" t="str">
+        <v>SENT</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Delivered via ICPaaS (Meta ID: wamid.HBgMOTE5Nzk1NjAwMjE3FQIAERgSOTNERUM5QTc5OTBBMDc4MTgzAA==)</v>
+      </c>
+      <c r="I3" t="str">
+        <v>23/10/2026, 3:33:03 pm</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>19</v>
+      <c r="B4" t="str">
+        <v>ADMIN PORTAL CONTROLLER</v>
       </c>
       <c r="C4">
         <v>918707744749</v>
       </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" t="s">
-        <v>22</v>
+      <c r="D4" t="str">
+        <v>PORTAL CONTROLLER</v>
+      </c>
+      <c r="E4" t="str">
+        <v>MEENA SHAH MEMORIAL SCHOOL</v>
+      </c>
+      <c r="F4" t="str">
+        <v>tabrezaalam92@gmail.com</v>
+      </c>
+      <c r="G4" t="str">
+        <v>SENT</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Delivered via ICPaaS (Meta ID: wamid.HBgMOTE4NzA3NzQ0NzQ5FQIAERgSNUJGQ0I0MjFFMjg2NDM0RkMxAA==)</v>
+      </c>
+      <c r="I4" t="str">
+        <v>23/10/2026, 3:33:03 pm</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>23</v>
+      <c r="B5" t="str">
+        <v>DR. RAMESH SHARMA</v>
       </c>
       <c r="C5">
         <v>919839012345</v>
       </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" t="s">
-        <v>26</v>
+      <c r="D5" t="str">
+        <v>SENIOR EVALUATOR</v>
+      </c>
+      <c r="E5" t="str">
+        <v>MEENA SHAH PUBLIC SCHOOL</v>
+      </c>
+      <c r="G5" t="str">
+        <v>SENT</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Delivered via ICPaaS (Meta ID: wamid.HBgMOTE5ODM5MDEyMzQ1FQIAERgSRDY5MkNBOEFFNkZBMDE5MDk4AA==)</v>
+      </c>
+      <c r="I5" t="str">
+        <v>23/10/2026, 3:33:03 pm</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>27</v>
+      <c r="B6" t="str">
+        <v>AJAY SIR</v>
       </c>
       <c r="C6">
         <v>919415534155</v>
       </c>
-      <c r="D6" t="s">
-        <v>28</v>
+      <c r="D6" t="str">
+        <v>DEAN MSITM COLLEGE</v>
+      </c>
+      <c r="G6" t="str">
+        <v>SENT</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Delivered via ICPaaS (Meta ID: wamid.HBgMOTE5NDE1NTM0MTU1FQIAERgSNTA2OEUxMDc2RkMxQzJGRjQ1AA==)</v>
+      </c>
+      <c r="I6" t="str">
+        <v>23/10/2026, 3:33:03 pm</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>29</v>
+      <c r="B7" t="str">
+        <v>SAEED SIR (baba ji)</v>
       </c>
       <c r="C7">
         <v>919839263821</v>
       </c>
-      <c r="D7" t="s">
-        <v>30</v>
+      <c r="D7" t="str">
+        <v>Manager</v>
+      </c>
+      <c r="G7" t="str">
+        <v>SENT</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Delivered via ICPaaS (Meta ID: wamid.HBgMOTE5ODM5MjYzODIxFQIAERgSM0M0NzI3ODM1ODk3QTE2MkY0AA==)</v>
+      </c>
+      <c r="I7" t="str">
+        <v>23/10/2026, 3:33:03 pm</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I7"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>